<commit_message>
Update Codal disclosure Excel report
</commit_message>
<xml_diff>
--- a/data/codal_disclosures_latest.xlsx
+++ b/data/codal_disclosures_latest.xlsx
@@ -480,7 +480,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T13:27:49+00:00</t>
+          <t>2026-10-13T13:29:16+00:00</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -797,7 +797,7 @@
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پارند_ثابت 🏛️ صندوق سرمایه گذاری پارند پایدار سپهر(ETF) 📋 تصمیمات مجمع صندوق سرمایه گذاری 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۵:۴۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 4 views 13:18 📋 اطلاعیه 📕 PDF</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پارند_ثابت 🏛️ صندوق سرمایه گذاری پارند پایدار سپهر(ETF) 📋 تصمیمات مجمع صندوق سرمایه گذاری 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۵:۴۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 5 views 13:18 📋 اطلاعیه 📕 PDF</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -847,7 +847,7 @@
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پاسا 🏛️ ایران یاسا تایر و رابر 📋 مشخصات کمیته ریسک 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۵:۳۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 4 views 13:18 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پاسا 🏛️ ایران یاسا تایر و رابر 📋 مشخصات کمیته ریسک 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۵:۳۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 5 views 13:18 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -897,7 +897,7 @@
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #ولملت 🏛️ واسپاری ملت 📋 توقف نماد معاملاتی ناشر به استناد ماده ۱۹ مکرر/ ۱۲ مکرر ۳دستورالعمل اجرایی نحوه انجام معاملات 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۲:۳۰ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 5 views 13:15 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #ولملت 🏛️ واسپاری ملت 📋 توقف نماد معاملاتی ناشر به استناد ماده ۱۹ مکرر/ ۱۲ مکرر ۳دستورالعمل اجرایی نحوه انجام معاملات 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۲:۳۰ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 6 views 13:15 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -947,7 +947,7 @@
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پاسا 🏛️ ایران یاسا تایر و رابر 📋 کمیته انتصابات 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۲:۲۴ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 5 views 13:15 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پاسا 🏛️ ایران یاسا تایر و رابر 📋 کمیته انتصابات 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۲:۲۴ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 6 views 13:15 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -1355,7 +1355,7 @@
       <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #کفرآور 🏛️ فرآورده های سیمان شرق 📌 #گزارش_فعالیت_هیئت_مدیره 📋 گزارش فعالیت هیئت مدیره دوره ۱۲ ماهه منتهی به ۱۴۰۵/۰۵/۳۱ 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۶:۴۳ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 11 views 12:57 📋 اطلاعیه 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #کفرآور 🏛️ فرآورده های سیمان شرق 📌 #گزارش_فعالیت_هیئت_مدیره 📋 گزارش فعالیت هیئت مدیره دوره ۱۲ ماهه منتهی به ۱۴۰۵/۰۵/۳۱ 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۶:۴۳ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 12 views 12:57 📋 اطلاعیه 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1409,7 +1409,7 @@
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پیمان 🏛️ پیمان غرب 📌 #توضیحات_در_خصوص_اطلاعات_و_صورت_های_مالی_منتشر_شده 📋 توضیحات در خصوص اطلاعات و صورت های مالی منتشر شده 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۴:۴۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 11 views 12:57 📋 اطلاعیه 📕 PDF</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پیمان 🏛️ پیمان غرب 📌 #توضیحات_در_خصوص_اطلاعات_و_صورت_های_مالی_منتشر_شده 📋 توضیحات در خصوص اطلاعات و صورت های مالی منتشر شده 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۴:۴۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 12 views 12:57 📋 اطلاعیه 📕 PDF</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #تپسی 🏛️ پیشگامان فن آوری و دانش آرامیس 📌 #مشخصات_کمیته_حسابرسی_و_واحد_حسابرسی_داخلی 📋 مشخصات کمیته حسابرسی و واحد حسابرسی داخلی 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۲:۳۰ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 11 views 12:54 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #تپسی 🏛️ پیشگامان فن آوری و دانش آرامیس 📌 #مشخصات_کمیته_حسابرسی_و_واحد_حسابرسی_داخلی 📋 مشخصات کمیته حسابرسی و واحد حسابرسی داخلی 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۲:۳۰ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 12 views 12:54 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -2267,7 +2267,7 @@
       <c r="H31" s="2" t="inlineStr"/>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #شپترو 🏛️ پتروشیمی آبادان 📋 مشخصات کمیته ریسک 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۵:۳۵:۱۳ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 13 views 12:06 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #شپترو 🏛️ پتروشیمی آبادان 📋 مشخصات کمیته ریسک 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۵:۳۵:۱۳ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 14 views 12:06 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2571,7 +2571,7 @@
       <c r="H37" s="2" t="inlineStr"/>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #فافق 🏛️ صنایع مس افق کرمان 📌 #معرفی /تغییر_در_ترکیب_اعضای_هیئت _مدیره 📋 معرفی /تغییر در ترکیب اعضای هیئت مدیره/مدیر عامل(اصلاحیه) 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۵:۱۴:۱۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 9 views 11:45 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #فافق 🏛️ صنایع مس افق کرمان 📌 #معرفی /تغییر_در_ترکیب_اعضای_هیئت _مدیره 📋 معرفی /تغییر در ترکیب اعضای هیئت مدیره/مدیر عامل(اصلاحیه) 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۵:۱۴:۱۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 10 views 11:45 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -8807,7 +8807,7 @@
       <c r="H159" s="2" t="inlineStr"/>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #واتی 🏛️ گروه سرمایه گذاری آتیه دماوند 📌 #افشای_اطلاعات_با_اهمیت 📋 افشای اطلاعات بااهمیت - (برگزاری مزایده - گروه ب) منتهی به سال مالی ۱۴۰۵/۰۹/۳۰ 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۵:۳۸ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 4 views 13:18 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #واتی 🏛️ گروه سرمایه گذاری آتیه دماوند 📌 #افشای_اطلاعات_با_اهمیت 📋 افشای اطلاعات بااهمیت - (برگزاری مزایده - گروه ب) منتهی به سال مالی ۱۴۰۵/۰۹/۳۰ 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۵:۳۸ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 5 views 13:18 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -8899,7 +8899,7 @@
       <c r="H161" s="2" t="inlineStr"/>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #آسود 🏛️ نهال آرمان اقتصاد 📋 صورت وضعیت پورتفوی صندوق سرمایه گذاری دوره ۱ ماهه منتهی به ۱۴۰۵/۰۷/۱۵ 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۳:۵۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 4 views 13:15 📋 اطلاعیه 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #آسود 🏛️ نهال آرمان اقتصاد 📋 صورت وضعیت پورتفوی صندوق سرمایه گذاری دوره ۱ ماهه منتهی به ۱۴۰۵/۰۷/۱۵ 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۳:۵۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 5 views 13:15 📋 اطلاعیه 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -8953,7 +8953,7 @@
       <c r="H162" s="2" t="inlineStr"/>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #وزمین 🏛️ بانک ایران زمین 📌 #صورت_های_مالی_میان_دوره_ای 📋 صورت های مالی سال مالی منتهی به ۱۴۰۴/۱۲/۲۹ (حسابرسی شده) (شرکت توسعه تجارت داتام) 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۵۴:۴۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 1 view 13:27 📋 اطلاعیه 📕 PDF 📘 Excel 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #وزمین 🏛️ بانک ایران زمین 📌 #صورت_های_مالی_میان_دوره_ای 📋 صورت های مالی سال مالی منتهی به ۱۴۰۴/۱۲/۲۹ (حسابرسی شده) (شرکت توسعه تجارت داتام) 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۵۴:۴۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 3 views 13:27 📋 اطلاعیه 📕 PDF 📘 Excel 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -9511,7 +9511,7 @@
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پیمان 🏛️ پیمان غرب 📌 #توضیحات_در_خصوص_اطلاعات_و_صورت_های_مالی_منتشر_شده 📋 توضیحات در خصوص اطلاعات و صورت های مالی منتشر شده 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۴:۴۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 11 views 12:57 📋 اطلاعیه 📕 PDF</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پیمان 🏛️ پیمان غرب 📌 #توضیحات_در_خصوص_اطلاعات_و_صورت_های_مالی_منتشر_شده 📋 توضیحات در خصوص اطلاعات و صورت های مالی منتشر شده 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۴:۴۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 12 views 12:57 📋 اطلاعیه 📕 PDF</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -11459,7 +11459,7 @@
       <c r="H40" s="2" t="inlineStr"/>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #وزمین 🏛️ بانک ایران زمین 📌 #صورت_های_مالی_میان_دوره_ای 📋 صورت های مالی سال مالی منتهی به ۱۴۰۴/۱۲/۲۹ (حسابرسی شده) (شرکت توسعه تجارت داتام) 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۵۴:۴۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 1 view 13:27 📋 اطلاعیه 📕 PDF 📘 Excel 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #وزمین 🏛️ بانک ایران زمین 📌 #صورت_های_مالی_میان_دوره_ای 📋 صورت های مالی سال مالی منتهی به ۱۴۰۴/۱۲/۲۹ (حسابرسی شده) (شرکت توسعه تجارت داتام) 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۵۴:۴۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 3 views 13:27 📋 اطلاعیه 📕 PDF 📘 Excel 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -11662,7 +11662,7 @@
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #تپسی 🏛️ پیشگامان فن آوری و دانش آرامیس 📌 #مشخصات_کمیته_حسابرسی_و_واحد_حسابرسی_داخلی 📋 مشخصات کمیته حسابرسی و واحد حسابرسی داخلی 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۲:۳۰ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 11 views 12:54 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #تپسی 🏛️ پیشگامان فن آوری و دانش آرامیس 📌 #مشخصات_کمیته_حسابرسی_و_واحد_حسابرسی_داخلی 📋 مشخصات کمیته حسابرسی و واحد حسابرسی داخلی 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۲:۳۰ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 12 views 12:54 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -11695,7 +11695,7 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پیمان 🏛️ پیمان غرب 📌 #توضیحات_در_خصوص_اطلاعات_و_صورت_های_مالی_منتشر_شده 📋 توضیحات در خصوص اطلاعات و صورت های مالی منتشر شده 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۴:۴۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 11 views 12:57 📋 اطلاعیه 📕 PDF</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پیمان 🏛️ پیمان غرب 📌 #توضیحات_در_خصوص_اطلاعات_و_صورت_های_مالی_منتشر_شده 📋 توضیحات در خصوص اطلاعات و صورت های مالی منتشر شده 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۴:۴۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 12 views 12:57 📋 اطلاعیه 📕 PDF</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -11728,7 +11728,7 @@
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #کفرآور 🏛️ فرآورده های سیمان شرق 📌 #گزارش_فعالیت_هیئت_مدیره 📋 گزارش فعالیت هیئت مدیره دوره ۱۲ ماهه منتهی به ۱۴۰۵/۰۵/۳۱ 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۶:۴۳ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 11 views 12:57 📋 اطلاعیه 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #کفرآور 🏛️ فرآورده های سیمان شرق 📌 #گزارش_فعالیت_هیئت_مدیره 📋 گزارش فعالیت هیئت مدیره دوره ۱۲ ماهه منتهی به ۱۴۰۵/۰۵/۳۱ 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۲۶:۴۳ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 12 views 12:57 📋 اطلاعیه 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11992,7 +11992,7 @@
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پاسا 🏛️ ایران یاسا تایر و رابر 📋 کمیته انتصابات 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۲:۲۴ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 5 views 13:15 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پاسا 🏛️ ایران یاسا تایر و رابر 📋 کمیته انتصابات 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۲:۲۴ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 6 views 13:15 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -12025,7 +12025,7 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #ولملت 🏛️ واسپاری ملت 📋 توقف نماد معاملاتی ناشر به استناد ماده ۱۹ مکرر/ ۱۲ مکرر ۳دستورالعمل اجرایی نحوه انجام معاملات 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۲:۳۰ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 5 views 13:15 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #ولملت 🏛️ واسپاری ملت 📋 توقف نماد معاملاتی ناشر به استناد ماده ۱۹ مکرر/ ۱۲ مکرر ۳دستورالعمل اجرایی نحوه انجام معاملات 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۲:۳۰ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 6 views 13:15 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -12058,7 +12058,7 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #آسود 🏛️ نهال آرمان اقتصاد 📋 صورت وضعیت پورتفوی صندوق سرمایه گذاری دوره ۱ ماهه منتهی به ۱۴۰۵/۰۷/۱۵ 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۳:۵۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 4 views 13:15 📋 اطلاعیه 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #آسود 🏛️ نهال آرمان اقتصاد 📋 صورت وضعیت پورتفوی صندوق سرمایه گذاری دوره ۱ ماهه منتهی به ۱۴۰۵/۰۷/۱۵ 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۳:۵۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 5 views 13:15 📋 اطلاعیه 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -12091,7 +12091,7 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پاسا 🏛️ ایران یاسا تایر و رابر 📋 مشخصات کمیته ریسک 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۵:۳۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 4 views 13:18 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پاسا 🏛️ ایران یاسا تایر و رابر 📋 مشخصات کمیته ریسک 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۵:۳۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 5 views 13:18 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -12124,7 +12124,7 @@
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #واتی 🏛️ گروه سرمایه گذاری آتیه دماوند 📌 #افشای_اطلاعات_با_اهمیت 📋 افشای اطلاعات بااهمیت - (برگزاری مزایده - گروه ب) منتهی به سال مالی ۱۴۰۵/۰۹/۳۰ 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۵:۳۸ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 4 views 13:18 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #واتی 🏛️ گروه سرمایه گذاری آتیه دماوند 📌 #افشای_اطلاعات_با_اهمیت 📋 افشای اطلاعات بااهمیت - (برگزاری مزایده - گروه ب) منتهی به سال مالی ۱۴۰۵/۰۹/۳۰ 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۵:۳۸ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 5 views 13:18 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -12157,7 +12157,7 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پارند_ثابت 🏛️ صندوق سرمایه گذاری پارند پایدار سپهر(ETF) 📋 تصمیمات مجمع صندوق سرمایه گذاری 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۵:۴۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 4 views 13:18 📋 اطلاعیه 📕 PDF</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #پارند_ثابت 🏛️ صندوق سرمایه گذاری پارند پایدار سپهر(ETF) 📋 تصمیمات مجمع صندوق سرمایه گذاری 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۴۵:۴۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 5 views 13:18 📋 اطلاعیه 📕 PDF</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -12190,7 +12190,7 @@
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #وزمین 🏛️ بانک ایران زمین 📌 #صورت_های_مالی_میان_دوره_ای 📋 صورت های مالی سال مالی منتهی به ۱۴۰۴/۱۲/۲۹ (حسابرسی شده) (شرکت توسعه تجارت داتام) 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۵۴:۴۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 1 view 13:27 📋 اطلاعیه 📕 PDF 📘 Excel 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #وزمین 🏛️ بانک ایران زمین 📌 #صورت_های_مالی_میان_دوره_ای 📋 صورت های مالی سال مالی منتهی به ۱۴۰۴/۱۲/۲۹ (حسابرسی شده) (شرکت توسعه تجارت داتام) 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۶:۵۴:۴۲ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 3 views 13:27 📋 اطلاعیه 📕 PDF 📘 Excel 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -12256,7 +12256,7 @@
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #فافق 🏛️ صنایع مس افق کرمان 📌 #معرفی /تغییر_در_ترکیب_اعضای_هیئت _مدیره 📋 معرفی /تغییر در ترکیب اعضای هیئت مدیره/مدیر عامل(اصلاحیه) 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۵:۱۴:۱۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 9 views 11:45 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #فافق 🏛️ صنایع مس افق کرمان 📌 #معرفی /تغییر_در_ترکیب_اعضای_هیئت _مدیره 📋 معرفی /تغییر در ترکیب اعضای هیئت مدیره/مدیر عامل(اصلاحیه) 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۵:۱۴:۱۷ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 10 views 11:45 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -12454,7 +12454,7 @@
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>اطلاعیه کدال | بورس تریدر 🏷️ #شپترو 🏛️ پتروشیمی آبادان 📋 مشخصات کمیته ریسک 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۵:۳۵:۱۳ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 13 views 12:06 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
+          <t>اطلاعیه کدال | بورس تریدر 🏷️ #شپترو 🏛️ پتروشیمی آبادان 📋 مشخصات کمیته ریسک 🔗 لینک اطلاعیه 📆 ۱۴۰۵/۰۷/۲۱ ۱۵:۳۵:۱۳ ━━━━━━━━━━━━━━━ 🌐 Bourse-Trader.ir 🆔 @CodalBourseTrader 14 views 12:06 📋 اطلاعیه 📕 PDF 🔗 TSETMC 📊 سابقه 📈 چارت</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -17001,7 +17001,7 @@
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
@@ -17076,7 +17076,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>000		https://excel.codal.ir/service/Excel/GetAll/JBsqvslfTvARtL61f2Wg9w%3d%3d/0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
@@ -17102,7 +17102,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>curl: (28) Failed to connect to excel.codal.ir port 443 after 7000 ms: Timeout was reached</t>
+          <t>curl: (28) Failed to connect to excel.codal.ir port 443 after 7001 ms: Timeout was reached</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -17124,7 +17124,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>000		https://excel.codal.ir/service/Excel/GetAll/J1aPpo73eSoo2Dong5HGyg%3d%3d/0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
@@ -17150,7 +17150,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>curl: (28) Failed to connect to excel.codal.ir port 443 after 7000 ms: Timeout was reached</t>
+          <t>curl: (28) Failed to connect to excel.codal.ir port 443 after 7001 ms: Timeout was reached</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -17172,7 +17172,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>000		https://excel.codal.ir/service/Excel/GetAll/r2RrHefXhTNZFw8HmjCTZQ%3d%3d/0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -17198,7 +17198,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>curl: (28) Failed to connect to excel.codal.ir port 443 after 7000 ms: Timeout was reached</t>
+          <t>curl: (28) Failed to connect to excel.codal.ir port 443 after 7002 ms: Timeout was reached</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -17302,7 +17302,7 @@
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
@@ -17402,7 +17402,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>159651</t>
+          <t>159652</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -17435,7 +17435,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>156543</t>
+          <t>156546</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -17468,7 +17468,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>157998</t>
+          <t>157996</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -17501,7 +17501,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>157131</t>
+          <t>157132</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -17534,7 +17534,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>156459</t>
+          <t>156458</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -17600,7 +17600,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>162019</t>
+          <t>162016</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -17633,7 +17633,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>168504</t>
+          <t>168505</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -17656,7 +17656,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>000		https://excel.codal.ir/service/Excel/GetAll/JBsqvslfTvARtL61f2Wg9w%3d%3d/0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -17672,7 +17672,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>curl: (28) Failed to connect to excel.codal.ir port 443 after 7000 ms: Timeout was reached</t>
+          <t>curl: (28) Failed to connect to excel.codal.ir port 443 after 7001 ms: Timeout was reached</t>
         </is>
       </c>
     </row>
@@ -17689,7 +17689,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>000		https://excel.codal.ir/service/Excel/GetAll/J1aPpo73eSoo2Dong5HGyg%3d%3d/0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
@@ -17705,7 +17705,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>curl: (28) Failed to connect to excel.codal.ir port 443 after 7000 ms: Timeout was reached</t>
+          <t>curl: (28) Failed to connect to excel.codal.ir port 443 after 7001 ms: Timeout was reached</t>
         </is>
       </c>
     </row>
@@ -17722,7 +17722,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>000		https://excel.codal.ir/service/Excel/GetAll/r2RrHefXhTNZFw8HmjCTZQ%3d%3d/0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -17738,7 +17738,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>curl: (28) Failed to connect to excel.codal.ir port 443 after 7000 ms: Timeout was reached</t>
+          <t>curl: (28) Failed to connect to excel.codal.ir port 443 after 7002 ms: Timeout was reached</t>
         </is>
       </c>
     </row>

</xml_diff>